<commit_message>
feat(finance): merge L&E cards, hide insights, customize Assets header theme, and update bank seeders
</commit_message>
<xml_diff>
--- a/backend/prisma/seed-data/depreciation.xlsx
+++ b/backend/prisma/seed-data/depreciation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rfadilla/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ATI-User\Downloads\PCMI-Apps\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB9D8B12-2F63-D94C-9D53-BD7169C92B57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6E2CDE58-AD86-4FBE-9116-47DF9733746C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="24000" xr2:uid="{C49568A5-158C-924F-8878-5D75329F86B5}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14914" xr2:uid="{C49568A5-158C-924F-8878-5D75329F86B5}"/>
   </bookViews>
   <sheets>
     <sheet name="Deprec 2025" sheetId="10" r:id="rId1"/>
@@ -882,28 +882,28 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A2:V147"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="10.8125" defaultRowHeight="15.45"/>
   <cols>
-    <col min="1" max="2" width="11.33203125" style="4" customWidth="1"/>
+    <col min="1" max="2" width="11.3125" style="4" customWidth="1"/>
     <col min="3" max="3" width="69" style="4" customWidth="1"/>
-    <col min="4" max="4" width="14.33203125" style="4" customWidth="1"/>
-    <col min="5" max="5" width="6.6640625" style="4" customWidth="1"/>
-    <col min="6" max="6" width="13.83203125" style="4" customWidth="1"/>
-    <col min="7" max="7" width="12.6640625" style="4" customWidth="1"/>
-    <col min="8" max="8" width="11.6640625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="14.3125" style="4" customWidth="1"/>
+    <col min="5" max="5" width="6.6875" style="4" customWidth="1"/>
+    <col min="6" max="6" width="13.8125" style="4" customWidth="1"/>
+    <col min="7" max="7" width="12.6875" style="4" customWidth="1"/>
+    <col min="8" max="8" width="11.6875" style="4" customWidth="1"/>
     <col min="9" max="9" width="12.5" style="4" customWidth="1"/>
-    <col min="10" max="10" width="12.6640625" style="4" customWidth="1"/>
+    <col min="10" max="10" width="12.6875" style="4" customWidth="1"/>
     <col min="11" max="11" width="12.5" style="4" customWidth="1"/>
-    <col min="12" max="12" width="12.83203125" style="4" customWidth="1"/>
-    <col min="13" max="13" width="13.1640625" style="4" customWidth="1"/>
+    <col min="12" max="12" width="12.8125" style="4" customWidth="1"/>
+    <col min="13" max="13" width="13.1875" style="4" customWidth="1"/>
     <col min="14" max="14" width="13" style="4" customWidth="1"/>
-    <col min="15" max="15" width="13.1640625" style="4" customWidth="1"/>
-    <col min="16" max="16" width="12.83203125" style="4" customWidth="1"/>
-    <col min="17" max="17" width="13.33203125" style="4" customWidth="1"/>
-    <col min="18" max="18" width="13.1640625" style="4" customWidth="1"/>
-    <col min="19" max="20" width="16.33203125" style="4" customWidth="1"/>
-    <col min="21" max="21" width="15.83203125" style="4" customWidth="1"/>
-    <col min="22" max="16384" width="10.83203125" style="4"/>
+    <col min="15" max="15" width="13.1875" style="4" customWidth="1"/>
+    <col min="16" max="16" width="12.8125" style="4" customWidth="1"/>
+    <col min="17" max="17" width="13.3125" style="4" customWidth="1"/>
+    <col min="18" max="18" width="13.1875" style="4" customWidth="1"/>
+    <col min="19" max="20" width="16.3125" style="4" customWidth="1"/>
+    <col min="21" max="21" width="15.8125" style="4" customWidth="1"/>
+    <col min="22" max="16384" width="10.8125" style="4"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:22">

</xml_diff>

<commit_message>
chore(seed): update seed data and equity seeder
</commit_message>
<xml_diff>
--- a/backend/prisma/seed-data/depreciation.xlsx
+++ b/backend/prisma/seed-data/depreciation.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ATI-User\Downloads\PCMI-Apps\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder (2)\new-cms\backend\prisma\seed-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6E2CDE58-AD86-4FBE-9116-47DF9733746C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14914" xr2:uid="{C49568A5-158C-924F-8878-5D75329F86B5}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17685"/>
   </bookViews>
   <sheets>
     <sheet name="Deprec 2025" sheetId="10" r:id="rId1"/>
@@ -18,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Deprec 2025'!$A$2:$U$107</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -376,14 +375,14 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="6">
-    <numFmt numFmtId="41" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="167" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="168" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="169" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="167" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="169" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -476,23 +475,23 @@
   </borders>
   <cellStyleXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="41" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="41" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="41" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="169" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
-    <xf numFmtId="41" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="41" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="169" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
@@ -500,16 +499,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
@@ -523,50 +522,50 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="3" applyFont="1"/>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="41" fontId="6" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="4" applyFont="1"/>
-    <xf numFmtId="41" fontId="6" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="4" applyFont="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="0" xfId="3" applyNumberFormat="1"/>
     <xf numFmtId="15" fontId="6" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="41" fontId="6" fillId="0" borderId="0" xfId="4" applyFont="1"/>
-    <xf numFmtId="41" fontId="7" fillId="0" borderId="0" xfId="4" applyFont="1"/>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="41" fontId="7" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="41" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="4" applyFont="1"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="4" applyFont="1"/>
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="20">
     <cellStyle name="Comma [0]" xfId="1" builtinId="6"/>
-    <cellStyle name="Comma [0] 2" xfId="4" xr:uid="{E206625D-CE92-B946-878E-6AA0829E898C}"/>
-    <cellStyle name="Comma [0] 2 2" xfId="12" xr:uid="{2A804006-5001-5049-84D3-FB258FE2E1AB}"/>
-    <cellStyle name="Comma [0] 2 3" xfId="5" xr:uid="{20A799B3-BE5A-964F-BE1E-1391E29E7052}"/>
-    <cellStyle name="Comma [0] 2 3 2" xfId="10" xr:uid="{6B5DF09C-6668-004E-832C-859692394773}"/>
-    <cellStyle name="Comma [0] 2 3 2 2" xfId="17" xr:uid="{2EC272E1-F154-DE4D-8FFC-1738E0F2B485}"/>
-    <cellStyle name="Comma [0] 3" xfId="9" xr:uid="{DCC47050-EC02-4040-8ED8-306B64C985B1}"/>
-    <cellStyle name="Comma [0] 4" xfId="16" xr:uid="{5B145FB2-4D0A-B249-B369-54ABF0C38C9B}"/>
-    <cellStyle name="Comma 2" xfId="6" xr:uid="{EAAE8118-4A1E-3049-ADC2-FB2BB5557A52}"/>
-    <cellStyle name="Comma 2 2" xfId="7" xr:uid="{B0896BE0-35A1-2F49-8BC0-6D90093B48F4}"/>
-    <cellStyle name="Comma 3" xfId="13" xr:uid="{D01750FA-08E4-0C47-9357-0F62E9D605A3}"/>
-    <cellStyle name="Comma 4" xfId="15" xr:uid="{A2EC2101-5781-AC44-BED5-F1BDBB670F1A}"/>
+    <cellStyle name="Comma [0] 2" xfId="4"/>
+    <cellStyle name="Comma [0] 2 2" xfId="12"/>
+    <cellStyle name="Comma [0] 2 3" xfId="5"/>
+    <cellStyle name="Comma [0] 2 3 2" xfId="10"/>
+    <cellStyle name="Comma [0] 2 3 2 2" xfId="17"/>
+    <cellStyle name="Comma [0] 3" xfId="9"/>
+    <cellStyle name="Comma [0] 4" xfId="16"/>
+    <cellStyle name="Comma 2" xfId="6"/>
+    <cellStyle name="Comma 2 2" xfId="7"/>
+    <cellStyle name="Comma 3" xfId="13"/>
+    <cellStyle name="Comma 4" xfId="15"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="2" xr:uid="{3B5401B9-DE75-EB48-9DE0-B2B7DAD183EC}"/>
-    <cellStyle name="Normal 2 2" xfId="8" xr:uid="{54DAEB53-87F6-084C-A87B-7176E7EB83C2}"/>
-    <cellStyle name="Normal 2 3" xfId="19" xr:uid="{FA86753D-0FFC-1948-8EF3-B2B2A5BEC3D7}"/>
-    <cellStyle name="Normal 3" xfId="14" xr:uid="{8B874317-EAD8-D042-9017-3A3DD28E4B28}"/>
-    <cellStyle name="Normal 3 4 2" xfId="11" xr:uid="{B424239B-ED7C-D142-AC4A-5D267E1997FC}"/>
-    <cellStyle name="Normal 3 6" xfId="3" xr:uid="{0DE30895-D5B6-4F42-8773-FC3E05E857CB}"/>
-    <cellStyle name="Normal 3 6 2" xfId="18" xr:uid="{8ECA74BB-2D76-474D-9277-CB573693B101}"/>
+    <cellStyle name="Normal 2" xfId="2"/>
+    <cellStyle name="Normal 2 2" xfId="8"/>
+    <cellStyle name="Normal 2 3" xfId="19"/>
+    <cellStyle name="Normal 3" xfId="14"/>
+    <cellStyle name="Normal 3 4 2" xfId="11"/>
+    <cellStyle name="Normal 3 6" xfId="3"/>
+    <cellStyle name="Normal 3 6 2" xfId="18"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -877,33 +876,33 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1692EEDF-8A16-3C46-A7B3-857B99C3D466}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A2:V147"/>
-  <sheetFormatPr defaultColWidth="10.8125" defaultRowHeight="15.45"/>
+  <sheetFormatPr defaultColWidth="10.77734375" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="2" width="11.3125" style="4" customWidth="1"/>
+    <col min="1" max="2" width="11.33203125" style="4" customWidth="1"/>
     <col min="3" max="3" width="69" style="4" customWidth="1"/>
-    <col min="4" max="4" width="14.3125" style="4" customWidth="1"/>
-    <col min="5" max="5" width="6.6875" style="4" customWidth="1"/>
-    <col min="6" max="6" width="13.8125" style="4" customWidth="1"/>
-    <col min="7" max="7" width="12.6875" style="4" customWidth="1"/>
-    <col min="8" max="8" width="11.6875" style="4" customWidth="1"/>
-    <col min="9" max="9" width="12.5" style="4" customWidth="1"/>
-    <col min="10" max="10" width="12.6875" style="4" customWidth="1"/>
-    <col min="11" max="11" width="12.5" style="4" customWidth="1"/>
-    <col min="12" max="12" width="12.8125" style="4" customWidth="1"/>
-    <col min="13" max="13" width="13.1875" style="4" customWidth="1"/>
+    <col min="4" max="4" width="14.33203125" style="4" customWidth="1"/>
+    <col min="5" max="5" width="6.6640625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="13.77734375" style="4" customWidth="1"/>
+    <col min="7" max="7" width="12.6640625" style="4" customWidth="1"/>
+    <col min="8" max="8" width="11.6640625" style="4" customWidth="1"/>
+    <col min="9" max="9" width="12.44140625" style="4" customWidth="1"/>
+    <col min="10" max="10" width="12.6640625" style="4" customWidth="1"/>
+    <col min="11" max="11" width="12.44140625" style="4" customWidth="1"/>
+    <col min="12" max="12" width="12.77734375" style="4" customWidth="1"/>
+    <col min="13" max="13" width="13.109375" style="4" customWidth="1"/>
     <col min="14" max="14" width="13" style="4" customWidth="1"/>
-    <col min="15" max="15" width="13.1875" style="4" customWidth="1"/>
-    <col min="16" max="16" width="12.8125" style="4" customWidth="1"/>
-    <col min="17" max="17" width="13.3125" style="4" customWidth="1"/>
-    <col min="18" max="18" width="13.1875" style="4" customWidth="1"/>
-    <col min="19" max="20" width="16.3125" style="4" customWidth="1"/>
-    <col min="21" max="21" width="15.8125" style="4" customWidth="1"/>
-    <col min="22" max="16384" width="10.8125" style="4"/>
+    <col min="15" max="15" width="13.109375" style="4" customWidth="1"/>
+    <col min="16" max="16" width="12.77734375" style="4" customWidth="1"/>
+    <col min="17" max="17" width="13.33203125" style="4" customWidth="1"/>
+    <col min="18" max="18" width="13.109375" style="4" customWidth="1"/>
+    <col min="19" max="20" width="16.33203125" style="4" customWidth="1"/>
+    <col min="21" max="21" width="15.77734375" style="4" customWidth="1"/>
+    <col min="22" max="16384" width="10.77734375" style="4"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:22">

</xml_diff>